<commit_message>
docs/app: the static app with the Summary's site rows in the calculators' color key
</commit_message>
<xml_diff>
--- a/docs/app/forms/easi/2026-10-23_EASI Calculator.xlsx
+++ b/docs/app/forms/easi/2026-10-23_EASI Calculator.xlsx
@@ -429,7 +429,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -528,12 +528,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF6F8FB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="46">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -1059,11 +1071,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="213">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="19" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1600,13 +1642,25 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="19" fillId="20" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="19" fillId="22" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="20" fillId="20" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="20" fillId="22" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="20" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="20" fillId="22" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" horizontal="center"/>
     </xf>
   </cellXfs>
@@ -22307,104 +22361,104 @@
     </row>
     <row r="2" ht="18" customHeight="1"/>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="199" t="inlineStr">
+      <c r="A3" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">Reach name</t>
         </is>
       </c>
-      <c r="B3" s="200" t="str">
+      <c r="B3" s="208" t="str">
         <f>IF(ISBLANK(Scenario!B2),"",Scenario!B2)</f>
         <v/>
       </c>
-      <c r="C3" s="200"/>
-      <c r="D3" s="200"/>
+      <c r="C3" s="208"/>
+      <c r="D3" s="208"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="199" t="inlineStr">
+      <c r="A4" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">Assessment tier</t>
         </is>
       </c>
-      <c r="B4" s="200" t="inlineStr">
+      <c r="B4" s="209" t="inlineStr">
         <is>
           <t xml:space="preserve">Screening</t>
         </is>
       </c>
-      <c r="C4" s="200"/>
-      <c r="D4" s="200"/>
+      <c r="C4" s="209"/>
+      <c r="D4" s="209"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="199" t="inlineStr">
+      <c r="A5" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">Reach length</t>
         </is>
       </c>
-      <c r="B5" s="200"/>
-      <c r="C5" s="200"/>
-      <c r="D5" s="200"/>
+      <c r="B5" s="207"/>
+      <c r="C5" s="207"/>
+      <c r="D5" s="207"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="199" t="inlineStr">
+      <c r="A6" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">Drainage area</t>
         </is>
       </c>
-      <c r="B6" s="200"/>
-      <c r="C6" s="200"/>
-      <c r="D6" s="200"/>
+      <c r="B6" s="207"/>
+      <c r="C6" s="207"/>
+      <c r="D6" s="207"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="199" t="inlineStr">
+      <c r="A7" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">Stream order (Strahler)</t>
         </is>
       </c>
-      <c r="B7" s="200"/>
-      <c r="C7" s="200"/>
-      <c r="D7" s="200"/>
+      <c r="B7" s="207"/>
+      <c r="C7" s="207"/>
+      <c r="D7" s="207"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="199" t="inlineStr">
+      <c r="A8" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">NARS-9 region</t>
         </is>
       </c>
-      <c r="B8" s="200" t="str">
+      <c r="B8" s="208" t="str">
         <f>IF(ISBLANK(Scenario!K3),"",Scenario!K3)</f>
         <v/>
       </c>
-      <c r="C8" s="200"/>
-      <c r="D8" s="200"/>
+      <c r="C8" s="208"/>
+      <c r="D8" s="208"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="199" t="inlineStr">
+      <c r="A9" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">EPA Level I ecoregion</t>
         </is>
       </c>
-      <c r="B9" s="200"/>
-      <c r="C9" s="200"/>
-      <c r="D9" s="200"/>
+      <c r="B9" s="207"/>
+      <c r="C9" s="207"/>
+      <c r="D9" s="207"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="199" t="inlineStr">
+      <c r="A10" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">EPA Level II ecoregion</t>
         </is>
       </c>
-      <c r="B10" s="200"/>
-      <c r="C10" s="200"/>
-      <c r="D10" s="200"/>
+      <c r="B10" s="207"/>
+      <c r="C10" s="207"/>
+      <c r="D10" s="207"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="199" t="inlineStr">
+      <c r="A11" s="206" t="inlineStr">
         <is>
           <t xml:space="preserve">EPA Level III ecoregion</t>
         </is>
       </c>
-      <c r="B11" s="200"/>
-      <c r="C11" s="200"/>
-      <c r="D11" s="200"/>
+      <c r="B11" s="207"/>
+      <c r="C11" s="207"/>
+      <c r="D11" s="207"/>
     </row>
     <row r="12" ht="18" customHeight="1"/>
     <row r="13" ht="28" customHeight="1">
@@ -22436,7 +22490,7 @@
           <t xml:space="preserve">ECI</t>
         </is>
       </c>
-      <c r="B16" s="206" t="str">
+      <c r="B16" s="210" t="str">
         <f>IF(ISNUMBER(Results!$D$30),Results!$D$30,"")</f>
         <v/>
       </c>
@@ -22447,7 +22501,7 @@
           <t xml:space="preserve">Physical</t>
         </is>
       </c>
-      <c r="B17" s="207" t="str">
+      <c r="B17" s="211" t="str">
         <f>IF(ISNUMBER(Results!$D$27),Results!$D$27,"")</f>
         <v/>
       </c>
@@ -22458,7 +22512,7 @@
           <t xml:space="preserve">Chemical</t>
         </is>
       </c>
-      <c r="B18" s="207" t="str">
+      <c r="B18" s="211" t="str">
         <f>IF(ISNUMBER(Results!$D$28),Results!$D$28,"")</f>
         <v/>
       </c>
@@ -22469,7 +22523,7 @@
           <t xml:space="preserve">Biological</t>
         </is>
       </c>
-      <c r="B19" s="207" t="str">
+      <c r="B19" s="211" t="str">
         <f>IF(ISNUMBER(Results!$D$29),Results!$D$29,"")</f>
         <v/>
       </c>
@@ -22488,7 +22542,7 @@
           <t xml:space="preserve">Catchment hydrology</t>
         </is>
       </c>
-      <c r="B21" s="208" t="str">
+      <c r="B21" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$13),Metrics!$B$13,"")</f>
         <v/>
       </c>
@@ -22499,7 +22553,7 @@
           <t xml:space="preserve">Surface water storage</t>
         </is>
       </c>
-      <c r="B22" s="208" t="str">
+      <c r="B22" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$25),Metrics!$B$25,"")</f>
         <v/>
       </c>
@@ -22510,7 +22564,7 @@
           <t xml:space="preserve">Reach inflow</t>
         </is>
       </c>
-      <c r="B23" s="208" t="str">
+      <c r="B23" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$35),Metrics!$B$35,"")</f>
         <v/>
       </c>
@@ -22521,7 +22575,7 @@
           <t xml:space="preserve">Streamflow regime</t>
         </is>
       </c>
-      <c r="B24" s="208" t="str">
+      <c r="B24" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$47),Metrics!$B$47,"")</f>
         <v/>
       </c>
@@ -22540,7 +22594,7 @@
           <t xml:space="preserve">Low flow and baseflow dynamics</t>
         </is>
       </c>
-      <c r="B26" s="208" t="str">
+      <c r="B26" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$60),Metrics!$B$60,"")</f>
         <v/>
       </c>
@@ -22551,7 +22605,7 @@
           <t xml:space="preserve">High flow dynamics</t>
         </is>
       </c>
-      <c r="B27" s="208" t="str">
+      <c r="B27" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$70),Metrics!$B$70,"")</f>
         <v/>
       </c>
@@ -22562,7 +22616,7 @@
           <t xml:space="preserve">Floodplain connectivity</t>
         </is>
       </c>
-      <c r="B28" s="208" t="str">
+      <c r="B28" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$82),Metrics!$B$82,"")</f>
         <v/>
       </c>
@@ -22573,7 +22627,7 @@
           <t xml:space="preserve">Hyporheic connectivity</t>
         </is>
       </c>
-      <c r="B29" s="208" t="str">
+      <c r="B29" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$95),Metrics!$B$95,"")</f>
         <v/>
       </c>
@@ -22592,7 +22646,7 @@
           <t xml:space="preserve">Channel evolution</t>
         </is>
       </c>
-      <c r="B31" s="208" t="str">
+      <c r="B31" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$109),Metrics!$B$109,"")</f>
         <v/>
       </c>
@@ -22603,7 +22657,7 @@
           <t xml:space="preserve">Channel and floodplain dynamics</t>
         </is>
       </c>
-      <c r="B32" s="208" t="str">
+      <c r="B32" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$121),Metrics!$B$121,"")</f>
         <v/>
       </c>
@@ -22614,7 +22668,7 @@
           <t xml:space="preserve">Sediment continuity</t>
         </is>
       </c>
-      <c r="B33" s="208" t="str">
+      <c r="B33" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$135),Metrics!$B$135,"")</f>
         <v/>
       </c>
@@ -22625,7 +22679,7 @@
           <t xml:space="preserve">Bed composition and large wood</t>
         </is>
       </c>
-      <c r="B34" s="208" t="str">
+      <c r="B34" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$145),Metrics!$B$145,"")</f>
         <v/>
       </c>
@@ -22644,7 +22698,7 @@
           <t xml:space="preserve">Light &amp; thermal regime</t>
         </is>
       </c>
-      <c r="B36" s="208" t="str">
+      <c r="B36" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$160),Metrics!$B$160,"")</f>
         <v/>
       </c>
@@ -22655,7 +22709,7 @@
           <t xml:space="preserve">Carbon processing</t>
         </is>
       </c>
-      <c r="B37" s="208" t="str">
+      <c r="B37" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$176),Metrics!$B$176,"")</f>
         <v/>
       </c>
@@ -22666,7 +22720,7 @@
           <t xml:space="preserve">Nutrient cycling</t>
         </is>
       </c>
-      <c r="B38" s="208" t="str">
+      <c r="B38" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$188),Metrics!$B$188,"")</f>
         <v/>
       </c>
@@ -22677,7 +22731,7 @@
           <t xml:space="preserve">Water &amp; soil quality</t>
         </is>
       </c>
-      <c r="B39" s="208" t="str">
+      <c r="B39" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$199),Metrics!$B$199,"")</f>
         <v/>
       </c>
@@ -22696,7 +22750,7 @@
           <t xml:space="preserve">Habitat provision</t>
         </is>
       </c>
-      <c r="B41" s="208" t="str">
+      <c r="B41" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$212),Metrics!$B$212,"")</f>
         <v/>
       </c>
@@ -22707,7 +22761,7 @@
           <t xml:space="preserve">Population support</t>
         </is>
       </c>
-      <c r="B42" s="208" t="str">
+      <c r="B42" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$225),Metrics!$B$225,"")</f>
         <v/>
       </c>
@@ -22718,7 +22772,7 @@
           <t xml:space="preserve">Community dynamics</t>
         </is>
       </c>
-      <c r="B43" s="208" t="str">
+      <c r="B43" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$235),Metrics!$B$235,"")</f>
         <v/>
       </c>
@@ -22729,7 +22783,7 @@
           <t xml:space="preserve">Watershed connectivity</t>
         </is>
       </c>
-      <c r="B44" s="208" t="str">
+      <c r="B44" s="212" t="str">
         <f>IF(ISNUMBER(Metrics!$B$245),Metrics!$B$245,"")</f>
         <v/>
       </c>

</xml_diff>